<commit_message>
Actualización preguntas de colores
</commit_message>
<xml_diff>
--- a/Juegos/General/cartas.xlsx
+++ b/Juegos/General/cartas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexa\Documents\IU digital\Aula juego\Dinamico\TwineJuegaboratorio\Juegos\General\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90FFB953-26EA-4F55-BB12-2AF5500EBABE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AFD6F02-EE41-4976-843A-88D9C8036437}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="83">
   <si>
     <t>Categoría</t>
   </si>
@@ -45,9 +45,6 @@
     <t>Física</t>
   </si>
   <si>
-    <t>¿Cuál es el color central del arcoiris?</t>
-  </si>
-  <si>
     <t>verde</t>
   </si>
   <si>
@@ -87,13 +84,7 @@
     <t>Rojo, Blanco</t>
   </si>
   <si>
-    <t>¿Qué color refleja la clorofila, el famoso pigmento que permite a las plantas atrapar la luz del sol para alimentarse?</t>
-  </si>
-  <si>
     <t>Los glóbulos rojos contienen hemoglobina, una proteína con hierro que se tiñe de este color al unirse al oxígeno. Los glóbulos blancos, que son nuestras células de defensa celular, no tienen este pigmento y por eso son pálidos.</t>
-  </si>
-  <si>
-    <t>Si miras un pingüino emperador, ¿qué tres colores destacan en sus plumas?</t>
   </si>
   <si>
     <t>Negro, Blanco, Amarillo</t>
@@ -134,18 +125,12 @@
     </r>
   </si>
   <si>
-    <t>¿De qué color es la obsidiana, esa roca de vidrio volcánico muy afilada que usaban las antiguas civilizaciones para hacer lanzas?</t>
-  </si>
-  <si>
     <t>Cuando la lava de un volcán se enfría tan rápido que no le da tiempo a formar cristales claros, atrapa minerales oscuros como el hierro y el magnesio, creando un vidrio liso y completamente negro.</t>
   </si>
   <si>
     <t>Amarillo</t>
   </si>
   <si>
-    <t>El azufre en su estado sólido natural forma cristales que, por su estructura atómica, absorben ciertos tonos de luz y reflejan un amarillo muy brillante y llamativo.</t>
-  </si>
-  <si>
     <t>Amarillo, Naranja, Rojo</t>
   </si>
   <si>
@@ -159,9 +144,6 @@
   </si>
   <si>
     <t>Se llama sistema RGB (Red, Green, Blue). Nuestros ojos tienen receptores sensibles exactamente a la luz roja, verde y azul. La pantalla engaña a nuestro cerebro mezclando estas tres luces para hacernos ver cualquier otro color.</t>
-  </si>
-  <si>
-    <t>Si miras el cielo con un telescopio, ¿de qué color se ven las estrellas que están muriendo y de qué color las más calientes y jóvenes?</t>
   </si>
   <si>
     <t>Azul, rojo</t>
@@ -253,22 +235,115 @@
 Lo vemos amarillo, naranja o rojo desde la Tierra debido a la atmósfera terrestre. Esta actúa como un filtro que dispersa las ondas de luz más cortas (como el azul y el violeta)</t>
   </si>
   <si>
-    <t>Cuando encuentras azufre puro cerca del cráter de un volcán, ¿de qué color es este mineral?</t>
-  </si>
-  <si>
     <t>La clorofila es excelente absorbiendo la luz en tonos rojos y azules para obtener energía, pero rebota o refleja la luz verde, que es la que finalmente llega a nuestros ojos.</t>
   </si>
   <si>
     <t>Si miras con una lupa muy potente la pantalla de tu celular, verás que todos los colores se crean mezclando solo tres luces primarias. ¿Cuáles son?</t>
   </si>
   <si>
-    <t>Cuando un objeto atrapa toda la luz que le llega y no refleja ni un solo rayo de luz hacia nuestros ojos, ¿de qué color lo vemos?</t>
-  </si>
-  <si>
     <t>El calor hace que los electrones del sodio salten. Cuando vuelven a su lugar, liberan esa energía sobrante en forma de luz. La cantidad de energía exacta que libera el sodio corresponde a la onda de luz amarilla.</t>
   </si>
   <si>
-    <t>Conocida como Luna de sangre. La atmósfera de la Tierra actúa como un lente que bloquea la luz azul del Sol pero deja pasar la luz roja (igual que en los atardeceres), proyectando ese tono sobre la Luna.</t>
+    <t>¿De qué color es Caño Cristales?</t>
+  </si>
+  <si>
+    <t>Rojo, Rosado, verde, amarillo, azul, negro</t>
+  </si>
+  <si>
+    <t>El efecto visual del arcoíris se forma por una combinación de factores biológicos y ambientales: plantas, musgos, algas,  arena dorada, el cuarzo y el hierro del lecho rocoso.</t>
+  </si>
+  <si>
+    <t>¿Cuál es el color que está en el centro del arcoiris?</t>
+  </si>
+  <si>
+    <t>¿Qué color refleja la clorofila, el pigmento que permite a las plantas atrapar la luz del sol para alimentarse?</t>
+  </si>
+  <si>
+    <t>Si miras un pingüino emperador, ¿qué colores destacan en sus plumas?</t>
+  </si>
+  <si>
+    <t>¿De qué color es la obsidiana, esa roca de vidrio volcánico muy afilada?</t>
+  </si>
+  <si>
+    <t>Si miras el cielo con un telescopio, ¿de qué color se ven las estrellas que están muriendo y de qué color las más jóvenes?</t>
+  </si>
+  <si>
+    <t>Cuando un objeto atrapa toda la luz y no refleja ni un solo rayo hacia nuestros ojos, ¿de qué color lo vemos?</t>
+  </si>
+  <si>
+    <t>Conocida como Luna de sangre. La atmósfera de la Tierra actúa como un lente que bloquea la luz azul del Sol pero deja pasar la luz roja, proyectando ese tono sobre la Luna.</t>
+  </si>
+  <si>
+    <t>u piel es totalmente negra para absorber y retener mejor el calor del sol en el extremo frío del Ártico. Además, su pelo no es blanco, es transparente y hueco; solo refleja la luz de la nieve.</t>
+  </si>
+  <si>
+    <t>¿De qué color eran las zanahorias silvestres originales?</t>
+  </si>
+  <si>
+    <t>¿De qué color es realmente la piel de un oso polar?</t>
+  </si>
+  <si>
+    <t>Morado</t>
+  </si>
+  <si>
+    <t>Las zanahorias antiguas eran moradas por fuera y amarillas por dentro. El tono naranja fue una mutación seleccionada artificialmente por los humanos.</t>
+  </si>
+  <si>
+    <t>¿Cuáles son los colores de una cebra bebé?</t>
+  </si>
+  <si>
+    <t>Café, blanco</t>
+  </si>
+  <si>
+    <t>Los potros de cebra nacen con rayas marrones que se van oscureciendo hasta volverse completamente negras a medida que crecen y maduran.</t>
+  </si>
+  <si>
+    <t>Los famosos cinco aros olímpicos están diseñados para representar la unión de los continentes. ¿Cuáles son los cinco colores de estos anillos?</t>
+  </si>
+  <si>
+    <t>Azul, Amarillo, Negro, Verde, Rojo</t>
+  </si>
+  <si>
+    <t>Cada aro representaba los colores de las banderas de los primeros países que tomaron parte de los JJ. OO</t>
+  </si>
+  <si>
+    <t>¿Cuáles son los cuatro colores que conforman las letras del logotipo de Google?</t>
+  </si>
+  <si>
+    <t>Azul, Rojo, Amarillo, Verde</t>
+  </si>
+  <si>
+    <t>Los diseñadores usaron los tres colores primarios (azul, rojo y amarillo) pero agregaron el verde en la letra l para demostrar que en Google no siguen las reglas tradicionales.</t>
+  </si>
+  <si>
+    <t>En el fútbol profesional, el árbitro tiene dos tarjetas en su bolsillo para castigar las faltas. ¿De qué colores son la de advertencia y la de expulsión?</t>
+  </si>
+  <si>
+    <t>Amarillo, Rojo</t>
+  </si>
+  <si>
+    <t>Se inventaron para el Mundial de 1970 con el fin de superar la barrera del idioma, inspirándose en los colores de los semáforos internacionales.</t>
+  </si>
+  <si>
+    <t>¿Cuáles son los dos colores que componen el logo oficial de la aplicación de mensajería WhatsApp?</t>
+  </si>
+  <si>
+    <t>Verde, Blanco</t>
+  </si>
+  <si>
+    <t>un globo de diálogo que indica comunicación y un teléfono antiguo adentro, usando el verde porque psicológicamente transmite seguridad y vía libre para hablar</t>
+  </si>
+  <si>
+    <t>Cultura general</t>
+  </si>
+  <si>
+    <t>Adquieren su característico color rosado o rojizo al cabo de unos años gracias a su alimentación, rica en crustáceos y algas que contienen unos pigmentos naturales</t>
+  </si>
+  <si>
+    <t>Blanco, Gris</t>
+  </si>
+  <si>
+    <t>¿De qué color son los flamencos al nacer?</t>
   </si>
 </sst>
 </file>
@@ -323,16 +398,16 @@
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -614,13 +689,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.85546875" style="1" customWidth="1"/>
     <col min="2" max="2" width="51.42578125" style="2" customWidth="1"/>
     <col min="3" max="3" width="28" style="1" customWidth="1"/>
-    <col min="4" max="4" width="24.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="24.7109375" style="2" customWidth="1"/>
     <col min="5" max="5" width="74.28515625" style="2" customWidth="1"/>
     <col min="6" max="16384" width="9.140625" style="1"/>
   </cols>
@@ -636,10 +711,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="45" x14ac:dyDescent="0.25">
@@ -647,16 +722,16 @@
         <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>6</v>
+        <v>52</v>
       </c>
       <c r="C2" s="2">
         <v>1</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="105" x14ac:dyDescent="0.25">
@@ -664,16 +739,16 @@
         <v>5</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C3" s="2">
         <v>6</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="45" x14ac:dyDescent="0.25">
@@ -681,50 +756,50 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C4" s="2">
         <v>1</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C5" s="2">
         <v>1</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C6" s="1">
         <v>1</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>16</v>
+      <c r="D6" s="2" t="s">
+        <v>15</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="45" x14ac:dyDescent="0.25">
@@ -732,16 +807,16 @@
         <v>3</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C7" s="1">
         <v>2</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>19</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="45" x14ac:dyDescent="0.25">
@@ -749,16 +824,16 @@
         <v>3</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>20</v>
+        <v>53</v>
       </c>
       <c r="C8" s="1">
         <v>1</v>
       </c>
-      <c r="D8" s="1" t="s">
-        <v>7</v>
+      <c r="D8" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="60" x14ac:dyDescent="0.25">
@@ -766,16 +841,16 @@
         <v>3</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>22</v>
+        <v>54</v>
       </c>
       <c r="C9" s="1">
         <v>3</v>
       </c>
-      <c r="D9" t="s">
-        <v>23</v>
+      <c r="D9" s="2" t="s">
+        <v>20</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="45" x14ac:dyDescent="0.25">
@@ -783,16 +858,16 @@
         <v>3</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C10" s="1">
         <v>2</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>26</v>
+      <c r="D10" s="2" t="s">
+        <v>23</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="45" x14ac:dyDescent="0.25">
@@ -800,16 +875,16 @@
         <v>4</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="C11" s="1">
         <v>1</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>40</v>
+      <c r="D11" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="45" x14ac:dyDescent="0.25">
@@ -817,33 +892,33 @@
         <v>4</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="C12" s="1">
-        <v>1</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>30</v>
+        <v>3</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="C13" s="1">
         <v>3</v>
       </c>
-      <c r="D13" s="1" t="s">
-        <v>32</v>
+      <c r="D13" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="45" x14ac:dyDescent="0.25">
@@ -851,84 +926,220 @@
         <v>5</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C14" s="1">
-        <v>3</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>35</v>
+        <v>2</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>32</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>37</v>
+        <v>57</v>
       </c>
       <c r="C15" s="1">
-        <v>2</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>39</v>
+        <v>1</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="C16" s="1">
         <v>1</v>
       </c>
-      <c r="D16" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>41</v>
+      <c r="D16" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C17" s="1">
         <v>1</v>
       </c>
-      <c r="D17" s="1" t="s">
-        <v>30</v>
+      <c r="D17" s="2" t="s">
+        <v>41</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>46</v>
+        <v>4</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="C18" s="1">
+        <v>6</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C19" s="1">
         <v>1</v>
       </c>
-      <c r="D18" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>57</v>
+      <c r="D19" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C20" s="1">
+        <v>1</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C21" s="1">
+        <v>2</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C22" s="1">
+        <v>5</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C23" s="1">
+        <v>4</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C24" s="1">
+        <v>2</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C25" s="1">
+        <v>2</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C26" s="1">
+        <v>2</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>